<commit_message>
Printing certificates for each sheet separately
</commit_message>
<xml_diff>
--- a/data/IT-куб.xlsx
+++ b/data/IT-куб.xlsx
@@ -5,11 +5,11 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\CertificateGenerator\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Python\CertGen\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9192" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9192" activeTab="9"/>
   </bookViews>
   <sheets>
     <sheet name="Кибергигиена" sheetId="16" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="30">
   <si>
     <t>patronymic</t>
   </si>
@@ -120,6 +120,9 @@
   </si>
   <si>
     <t>Мобильная разработка</t>
+  </si>
+  <si>
+    <t>летние смены</t>
   </si>
 </sst>
 </file>
@@ -616,7 +619,7 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
-            <xm:f>cert_data!$A$1:$A$2</xm:f>
+            <xm:f>cert_data!$A$1:$A$3</xm:f>
           </x14:formula1>
           <xm:sqref>G2</xm:sqref>
         </x14:dataValidation>
@@ -671,7 +674,9 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" s="11"/>
+      <c r="A3" s="9" t="s">
+        <v>29</v>
+      </c>
       <c r="B3" s="10" t="s">
         <v>6</v>
       </c>
@@ -766,7 +771,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="Iz9XpwAHqxcpehazFnKokvtbK9GrewYjTCHG0Po8jGjFw+ZgyH0jod5ZWUC0wBJCJ+SfOCgoS+ZUkfrX3izONA==" saltValue="P8CN7ocJ138vUTRXYJNEbg==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="0HwJdK5vNqUg+cqBhJAh1yF2wwh8voqKX19ZHRz8nDQ7iB/+VVecZEGFIdZ6RfmOj6QgeU3q+Ax689hioyek8A==" saltValue="Ij26Fkyc8+SQFvBvwb+/WA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <sortState ref="C11:C15">
     <sortCondition ref="C11"/>
   </sortState>
@@ -839,21 +844,21 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
-            <xm:f>cert_data!$A$1:$A$2</xm:f>
+            <xm:f>cert_data!$B$1:$B$4</xm:f>
+          </x14:formula1>
+          <xm:sqref>E2</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>cert_data!$C$1:$C$15</xm:f>
+          </x14:formula1>
+          <xm:sqref>D2</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>cert_data!$A$1:$A$3</xm:f>
           </x14:formula1>
           <xm:sqref>G2</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
-          <x14:formula1>
-            <xm:f>cert_data!$B$1:$B$4</xm:f>
-          </x14:formula1>
-          <xm:sqref>E2</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
-          <x14:formula1>
-            <xm:f>cert_data!$C$1:$C$15</xm:f>
-          </x14:formula1>
-          <xm:sqref>D2</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -931,15 +936,15 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
-            <xm:f>cert_data!$A$1:$A$2</xm:f>
+            <xm:f>cert_data!$C$1:$C$15</xm:f>
+          </x14:formula1>
+          <xm:sqref>D2</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>cert_data!$A$1:$A$3</xm:f>
           </x14:formula1>
           <xm:sqref>G2</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
-          <x14:formula1>
-            <xm:f>cert_data!$C$1:$C$15</xm:f>
-          </x14:formula1>
-          <xm:sqref>D2</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1017,15 +1022,15 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
-            <xm:f>cert_data!$A$1:$A$2</xm:f>
+            <xm:f>cert_data!$C$1:$C$15</xm:f>
+          </x14:formula1>
+          <xm:sqref>D2</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>cert_data!$A$1:$A$3</xm:f>
           </x14:formula1>
           <xm:sqref>G2</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
-          <x14:formula1>
-            <xm:f>cert_data!$C$1:$C$15</xm:f>
-          </x14:formula1>
-          <xm:sqref>D2</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1103,15 +1108,15 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
-            <xm:f>cert_data!$A$1:$A$2</xm:f>
+            <xm:f>cert_data!$C$1:$C$15</xm:f>
+          </x14:formula1>
+          <xm:sqref>D2</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>cert_data!$A$1:$A$3</xm:f>
           </x14:formula1>
           <xm:sqref>G2</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
-          <x14:formula1>
-            <xm:f>cert_data!$C$1:$C$15</xm:f>
-          </x14:formula1>
-          <xm:sqref>D2</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1183,21 +1188,21 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
-            <xm:f>cert_data!$A$1:$A$2</xm:f>
+            <xm:f>cert_data!$B$1:$B$4</xm:f>
+          </x14:formula1>
+          <xm:sqref>E2</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>cert_data!$C$1:$C$15</xm:f>
+          </x14:formula1>
+          <xm:sqref>D2</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>cert_data!$A$1:$A$3</xm:f>
           </x14:formula1>
           <xm:sqref>G2</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
-          <x14:formula1>
-            <xm:f>cert_data!$B$1:$B$4</xm:f>
-          </x14:formula1>
-          <xm:sqref>E2</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
-          <x14:formula1>
-            <xm:f>cert_data!$C$1:$C$15</xm:f>
-          </x14:formula1>
-          <xm:sqref>D2</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1269,21 +1274,21 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
-            <xm:f>cert_data!$A$1:$A$2</xm:f>
+            <xm:f>cert_data!$B$1:$B$4</xm:f>
+          </x14:formula1>
+          <xm:sqref>E2</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>cert_data!$C$1:$C$15</xm:f>
+          </x14:formula1>
+          <xm:sqref>D2</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>cert_data!$A$1:$A$3</xm:f>
           </x14:formula1>
           <xm:sqref>G2</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
-          <x14:formula1>
-            <xm:f>cert_data!$B$1:$B$4</xm:f>
-          </x14:formula1>
-          <xm:sqref>E2</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
-          <x14:formula1>
-            <xm:f>cert_data!$C$1:$C$15</xm:f>
-          </x14:formula1>
-          <xm:sqref>D2</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1355,21 +1360,21 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="3">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
-            <xm:f>cert_data!$A$1:$A$2</xm:f>
+            <xm:f>cert_data!$B$1:$B$4</xm:f>
+          </x14:formula1>
+          <xm:sqref>E2</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>cert_data!$C$1:$C$15</xm:f>
+          </x14:formula1>
+          <xm:sqref>D2</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>cert_data!$A$1:$A$3</xm:f>
           </x14:formula1>
           <xm:sqref>G2</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
-          <x14:formula1>
-            <xm:f>cert_data!$B$1:$B$4</xm:f>
-          </x14:formula1>
-          <xm:sqref>E2</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
-          <x14:formula1>
-            <xm:f>cert_data!$C$1:$C$15</xm:f>
-          </x14:formula1>
-          <xm:sqref>D2</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1447,15 +1452,15 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
-            <xm:f>cert_data!$A$1:$A$2</xm:f>
+            <xm:f>cert_data!$C$1:$C$15</xm:f>
+          </x14:formula1>
+          <xm:sqref>D2</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>cert_data!$A$1:$A$3</xm:f>
           </x14:formula1>
           <xm:sqref>G2</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
-          <x14:formula1>
-            <xm:f>cert_data!$C$1:$C$15</xm:f>
-          </x14:formula1>
-          <xm:sqref>D2</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
Implemented a selection of sheets for printing
</commit_message>
<xml_diff>
--- a/data/IT-куб.xlsx
+++ b/data/IT-куб.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9192" activeTab="9"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="9192" activeTab="4"/>
   </bookViews>
   <sheets>
     <sheet name="Кибергигиена" sheetId="16" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="121" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="41">
   <si>
     <t>patronymic</t>
   </si>
@@ -123,6 +123,39 @@
   </si>
   <si>
     <t>летние смены</t>
+  </si>
+  <si>
+    <t>Иванов</t>
+  </si>
+  <si>
+    <t>Иван</t>
+  </si>
+  <si>
+    <t>Иванович</t>
+  </si>
+  <si>
+    <t>Петров</t>
+  </si>
+  <si>
+    <t>Петрович</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Пётр</t>
+  </si>
+  <si>
+    <t>Сергеев</t>
+  </si>
+  <si>
+    <t>Сергей</t>
+  </si>
+  <si>
+    <t>Сергеевич</t>
+  </si>
+  <si>
+    <t>Дроздов</t>
+  </si>
+  <si>
+    <t>Никитич</t>
   </si>
 </sst>
 </file>
@@ -597,20 +630,30 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
+      <c r="A2" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>32</v>
+      </c>
       <c r="D2" s="6" t="s">
         <v>7</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F2" s="3"/>
+      <c r="F2" s="3">
+        <v>144</v>
+      </c>
       <c r="G2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="H2" s="2"/>
+      <c r="H2" s="2">
+        <v>112</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -822,20 +865,30 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
+      <c r="A2" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>34</v>
+      </c>
       <c r="D2" s="6" t="s">
         <v>17</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="F2" s="3"/>
+      <c r="F2" s="3">
+        <v>144</v>
+      </c>
       <c r="G2" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="H2" s="2"/>
+        <v>9</v>
+      </c>
+      <c r="H2" s="2">
+        <v>113</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -908,20 +961,30 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
+      <c r="A2" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>38</v>
+      </c>
       <c r="D2" s="6" t="s">
         <v>18</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F2" s="3"/>
+      <c r="F2" s="3">
+        <v>136</v>
+      </c>
       <c r="G2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="H2" s="2"/>
+      <c r="H2" s="2">
+        <v>155</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1080,20 +1143,30 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="12"/>
-      <c r="B2" s="12"/>
-      <c r="C2" s="12"/>
+      <c r="A2" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="12" t="s">
+        <v>40</v>
+      </c>
       <c r="D2" s="6" t="s">
         <v>28</v>
       </c>
       <c r="E2" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="F2" s="3"/>
+      <c r="F2" s="3">
+        <v>144</v>
+      </c>
       <c r="G2" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="H2" s="2"/>
+      <c r="H2" s="2">
+        <v>567</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>